<commit_message>
added new quizzes to the gridReveal...
</commit_message>
<xml_diff>
--- a/public/gameSources/gridReveal/gameData/quiz-data.xlsx
+++ b/public/gameSources/gridReveal/gameData/quiz-data.xlsx
@@ -8,14 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\charlie\Desktop\gridReveal\public\gameData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBBF9F50-CA85-4C26-BAA5-9A0D4D75DF85}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13A9BDD4-5B8E-43DD-AD48-CCC421578D2B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="g1-general-knowledge" sheetId="6" r:id="rId1"/>
     <sheet name="g3-system-unit" sheetId="7" r:id="rId2"/>
     <sheet name="g5-computer-network" sheetId="8" r:id="rId3"/>
+    <sheet name="g2-parts-of-a-computer" sheetId="9" r:id="rId4"/>
+    <sheet name="kg-computer-parts" sheetId="10" r:id="rId5"/>
+    <sheet name="g5-types-of-network" sheetId="11" r:id="rId6"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -27,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="200">
   <si>
     <t>Questions</t>
   </si>
@@ -411,6 +414,222 @@
   </si>
   <si>
     <t>False</t>
+  </si>
+  <si>
+    <t>Parts of A Computer</t>
+  </si>
+  <si>
+    <t>https://i.pinimg.com/736x/72/43/a1/7243a1c0cfbe9d859af4ce4770981099.jpg</t>
+  </si>
+  <si>
+    <t>To learn about the basic parts of a computer</t>
+  </si>
+  <si>
+    <t>Monitor</t>
+  </si>
+  <si>
+    <t>Keyboard</t>
+  </si>
+  <si>
+    <t>Mouse</t>
+  </si>
+  <si>
+    <t>Speaker</t>
+  </si>
+  <si>
+    <t>Printer</t>
+  </si>
+  <si>
+    <t>WebCam</t>
+  </si>
+  <si>
+    <t>Scanner</t>
+  </si>
+  <si>
+    <t>Game Controller</t>
+  </si>
+  <si>
+    <t>You can type using a CPU.</t>
+  </si>
+  <si>
+    <t>CPU is a processing device.</t>
+  </si>
+  <si>
+    <t>Keyboard is an input device.</t>
+  </si>
+  <si>
+    <t>Monitor is an output device.</t>
+  </si>
+  <si>
+    <t>You can watch movies on a monitor.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">You can use a mouse to draw pictures on a computer. </t>
+  </si>
+  <si>
+    <t>What's the brain of a computer?</t>
+  </si>
+  <si>
+    <t>CPU stands for________.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">You can hear souds from speakers. </t>
+  </si>
+  <si>
+    <t>What do you use to print pictures and text on paper?</t>
+  </si>
+  <si>
+    <t>Central Processing Unit</t>
+  </si>
+  <si>
+    <t>A printer.</t>
+  </si>
+  <si>
+    <t>https://media.baamboozle.com/uploads/images/1392941/4e187cd8-d2de-4292-9926-3b707c137548.gif</t>
+  </si>
+  <si>
+    <t>https://media.baamboozle.com/uploads/images/1392941/58d855af-4b4e-437e-b145-18401715842e-thumbnail.jpeg</t>
+  </si>
+  <si>
+    <t>https://media.baamboozle.com/uploads/images/1392941/e2e37a00-4bec-4746-81d4-7f826c189807.jpeg</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn0.gstatic.com/images?q=tbn:ANd9GcRpt0gjitTiGYcFr-XsmHfx1jN3hAdrkmdQhCo2EBODhw&amp;s=10</t>
+  </si>
+  <si>
+    <t>https://www.projectaudio.com.au/cdn/shop/files/SpeakerBox3ECarbonBlack_1200x1200.png?v=1717660527</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn0.gstatic.com/images?q=tbn:ANd9GcQl2NOUFwA-71ZHIboNwo4cgnvZziVkfF8mwMWCi_nrqA&amp;s=10</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn0.gstatic.com/images?q=tbn:ANd9GcQnmlYYWXgiDRm5-lv8BS3uUhBL2zGTXFXSkhv38y8lNA&amp;s=10</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn0.gstatic.com/images?q=tbn:ANd9GcQoktFTYoiXkD1jSU97co_WsBYBOTTY2wu-vZyyCCr1JA&amp;s=10</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn0.gstatic.com/images?q=tbn:ANd9GcQfjNLRAy-Rj73hCS6yxYod35ZHDi4xDQD8NNEL8oAHBw&amp;s=10</t>
+  </si>
+  <si>
+    <t>KG</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn0.gstatic.com/images?q=tbn:ANd9GcSWozCeWHLVKGDgB3VPuBwC3MrrjlB-sQOAvU-dJ37vGeMWyLnbzVh9sXXh&amp;s=10</t>
+  </si>
+  <si>
+    <t>Computer is a machine.</t>
+  </si>
+  <si>
+    <t>What do we use to type letters and numbers?</t>
+  </si>
+  <si>
+    <t>What do we use to draw on a computer?</t>
+  </si>
+  <si>
+    <t>What is the brain of a computer?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">We can use that to see pictures and videos. </t>
+  </si>
+  <si>
+    <t>We use that to print pictures and stickers on paper.</t>
+  </si>
+  <si>
+    <t>We use that to hear sounds from a computer.</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn0.gstatic.com/images?q=tbn:ANd9GcQmMsg5FcEuw_VBGuFodHI_FuOIMTcgZnraSYAW22EWz0ulQsX0ZCW2cWmk&amp;s=10</t>
+  </si>
+  <si>
+    <t>Types of Computer Network</t>
+  </si>
+  <si>
+    <t>To learn about different types of computer network</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn0.gstatic.com/images?q=tbn:ANd9GcTTmsulqgSmJyazJUl5iyap78OchupQWuK0mktBAGHqpdduQ7lMofal03ci&amp;s=10</t>
+  </si>
+  <si>
+    <t>PAN stands for _____________.</t>
+  </si>
+  <si>
+    <t>LAN stands for _____________.</t>
+  </si>
+  <si>
+    <t>MAN stands for _____________.</t>
+  </si>
+  <si>
+    <t>WAN stands for _____________.</t>
+  </si>
+  <si>
+    <t>Name one communication channel used in a PAN network.</t>
+  </si>
+  <si>
+    <t>Name one communication channel used in a LAN network.</t>
+  </si>
+  <si>
+    <t>Name one communication channel used in a MAN network.</t>
+  </si>
+  <si>
+    <t>Name one communication channel used in a WAN network.</t>
+  </si>
+  <si>
+    <t>The Internet is the best example of a ____________ network.</t>
+  </si>
+  <si>
+    <t>If computers and devices are interconnected over a small area, it forms a _________ network.</t>
+  </si>
+  <si>
+    <t>If computers and devices are interconnected in the same office or building, it forms a _________ network.</t>
+  </si>
+  <si>
+    <t>If computers are interconnected over an entire city, it forms a ___________ network.</t>
+  </si>
+  <si>
+    <t>If computers are interconnected all over the world, it forms a _____________ network.</t>
+  </si>
+  <si>
+    <t>A collection of computers connected together is called a _____________.</t>
+  </si>
+  <si>
+    <t>Local Area Network</t>
+  </si>
+  <si>
+    <t>Metropolitan Area Network</t>
+  </si>
+  <si>
+    <t>Wide Area Network</t>
+  </si>
+  <si>
+    <t>Bluetooth/ WiFi</t>
+  </si>
+  <si>
+    <t>WiFi/Cables</t>
+  </si>
+  <si>
+    <t>Cables/Satellites</t>
+  </si>
+  <si>
+    <t>Satellites/ Fiber Optics Cables</t>
+  </si>
+  <si>
+    <t>WAN</t>
+  </si>
+  <si>
+    <t>PAN</t>
+  </si>
+  <si>
+    <t>LAN</t>
+  </si>
+  <si>
+    <t>MAN</t>
+  </si>
+  <si>
+    <t>computer network</t>
+  </si>
+  <si>
+    <t>Personal Area Network</t>
   </si>
 </sst>
 </file>
@@ -534,9 +753,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -553,6 +769,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -847,11 +1066,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" s="1" customFormat="1" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="17" t="s">
         <v>77</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
     </row>
     <row r="2" spans="1:5" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
@@ -894,8 +1113,8 @@
       <c r="C5" s="4"/>
     </row>
     <row r="6" spans="1:5" s="7" customFormat="1" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="13"/>
-      <c r="B6" s="13"/>
+      <c r="A6" s="12"/>
+      <c r="B6" s="12"/>
       <c r="C6" s="8"/>
       <c r="D6" s="6"/>
       <c r="E6" s="6"/>
@@ -910,21 +1129,21 @@
       <c r="C7" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="D7" s="12" t="s">
+      <c r="D7" s="11" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="3.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="14" t="s">
+      <c r="A8" s="13" t="s">
         <v>73</v>
       </c>
-      <c r="B8" s="14" t="s">
+      <c r="B8" s="13" t="s">
         <v>74</v>
       </c>
-      <c r="C8" s="14" t="s">
+      <c r="C8" s="13" t="s">
         <v>75</v>
       </c>
-      <c r="D8" s="15" t="s">
+      <c r="D8" s="14" t="s">
         <v>76</v>
       </c>
     </row>
@@ -938,7 +1157,7 @@
       <c r="C9" s="10">
         <v>15</v>
       </c>
-      <c r="D9" s="16" t="s">
+      <c r="D9" s="15" t="s">
         <v>68</v>
       </c>
       <c r="E9" s="2"/>
@@ -1735,11 +1954,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" s="1" customFormat="1" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="17" t="s">
         <v>77</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
     </row>
     <row r="2" spans="1:5" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
@@ -1782,8 +2001,8 @@
       <c r="C5" s="4"/>
     </row>
     <row r="6" spans="1:5" s="7" customFormat="1" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="13"/>
-      <c r="B6" s="13"/>
+      <c r="A6" s="12"/>
+      <c r="B6" s="12"/>
       <c r="C6" s="8"/>
       <c r="D6" s="6"/>
       <c r="E6" s="6"/>
@@ -1798,21 +2017,21 @@
       <c r="C7" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="D7" s="12" t="s">
+      <c r="D7" s="11" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="3.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="14" t="s">
+      <c r="A8" s="13" t="s">
         <v>73</v>
       </c>
-      <c r="B8" s="14" t="s">
+      <c r="B8" s="13" t="s">
         <v>74</v>
       </c>
-      <c r="C8" s="14" t="s">
+      <c r="C8" s="13" t="s">
         <v>75</v>
       </c>
-      <c r="D8" s="15" t="s">
+      <c r="D8" s="14" t="s">
         <v>76</v>
       </c>
     </row>
@@ -1820,13 +2039,13 @@
       <c r="A9" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="B9" s="17" t="s">
+      <c r="B9" s="16" t="s">
         <v>84</v>
       </c>
       <c r="C9" s="10">
         <v>15</v>
       </c>
-      <c r="D9" s="16" t="s">
+      <c r="D9" s="15" t="s">
         <v>100</v>
       </c>
       <c r="E9" s="2"/>
@@ -1835,7 +2054,7 @@
       <c r="A10" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="B10" s="17" t="s">
+      <c r="B10" s="16" t="s">
         <v>84</v>
       </c>
       <c r="C10" s="10">
@@ -1850,7 +2069,7 @@
       <c r="A11" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="B11" s="17" t="s">
+      <c r="B11" s="16" t="s">
         <v>86</v>
       </c>
       <c r="C11" s="10">
@@ -1865,7 +2084,7 @@
       <c r="A12" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="B12" s="17" t="s">
+      <c r="B12" s="16" t="s">
         <v>87</v>
       </c>
       <c r="C12" s="10">
@@ -1880,7 +2099,7 @@
       <c r="A13" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="B13" s="17" t="s">
+      <c r="B13" s="16" t="s">
         <v>88</v>
       </c>
       <c r="C13" s="10">
@@ -1895,7 +2114,7 @@
       <c r="A14" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="B14" s="17" t="s">
+      <c r="B14" s="16" t="s">
         <v>89</v>
       </c>
       <c r="C14" s="10">
@@ -1910,7 +2129,7 @@
       <c r="A15" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="B15" s="17" t="s">
+      <c r="B15" s="16" t="s">
         <v>90</v>
       </c>
       <c r="C15" s="10">
@@ -1925,7 +2144,7 @@
       <c r="A16" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="B16" s="17" t="s">
+      <c r="B16" s="16" t="s">
         <v>91</v>
       </c>
       <c r="C16" s="10">
@@ -1940,7 +2159,7 @@
       <c r="A17" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="B17" s="17" t="s">
+      <c r="B17" s="16" t="s">
         <v>92</v>
       </c>
       <c r="C17" s="10">
@@ -1955,7 +2174,7 @@
       <c r="A18" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="B18" s="17" t="s">
+      <c r="B18" s="16" t="s">
         <v>126</v>
       </c>
       <c r="C18" s="10">
@@ -1968,7 +2187,7 @@
       <c r="A19" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="B19" s="17" t="s">
+      <c r="B19" s="16" t="s">
         <v>126</v>
       </c>
       <c r="C19" s="10">
@@ -1981,7 +2200,7 @@
       <c r="A20" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="B20" s="17" t="s">
+      <c r="B20" s="16" t="s">
         <v>127</v>
       </c>
       <c r="C20" s="10">
@@ -1994,7 +2213,7 @@
       <c r="A21" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="B21" s="17" t="s">
+      <c r="B21" s="16" t="s">
         <v>90</v>
       </c>
       <c r="C21" s="10">
@@ -2007,7 +2226,7 @@
       <c r="A22" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="B22" s="17" t="s">
+      <c r="B22" s="16" t="s">
         <v>89</v>
       </c>
       <c r="C22" s="10">
@@ -2020,7 +2239,7 @@
       <c r="A23" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="B23" s="17" t="s">
+      <c r="B23" s="16" t="s">
         <v>92</v>
       </c>
       <c r="C23" s="10">
@@ -2033,7 +2252,7 @@
       <c r="A24" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="B24" s="17" t="s">
+      <c r="B24" s="16" t="s">
         <v>91</v>
       </c>
       <c r="C24" s="10">
@@ -2552,11 +2771,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" s="1" customFormat="1" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="17" t="s">
         <v>77</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
     </row>
     <row r="2" spans="1:5" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
@@ -2599,8 +2818,8 @@
       <c r="C5" s="4"/>
     </row>
     <row r="6" spans="1:5" s="7" customFormat="1" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="13"/>
-      <c r="B6" s="13"/>
+      <c r="A6" s="12"/>
+      <c r="B6" s="12"/>
       <c r="C6" s="8"/>
       <c r="D6" s="6"/>
       <c r="E6" s="6"/>
@@ -2615,21 +2834,21 @@
       <c r="C7" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="D7" s="12" t="s">
+      <c r="D7" s="11" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="3.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="14" t="s">
+      <c r="A8" s="13" t="s">
         <v>73</v>
       </c>
-      <c r="B8" s="14" t="s">
+      <c r="B8" s="13" t="s">
         <v>74</v>
       </c>
-      <c r="C8" s="14" t="s">
+      <c r="C8" s="13" t="s">
         <v>75</v>
       </c>
-      <c r="D8" s="15" t="s">
+      <c r="D8" s="14" t="s">
         <v>76</v>
       </c>
     </row>
@@ -2637,20 +2856,20 @@
       <c r="A9" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="B9" s="17" t="s">
+      <c r="B9" s="16" t="s">
         <v>126</v>
       </c>
       <c r="C9" s="10">
         <v>15</v>
       </c>
-      <c r="D9" s="16"/>
+      <c r="D9" s="15"/>
       <c r="E9" s="2"/>
     </row>
     <row r="10" spans="1:5" s="9" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="B10" s="17" t="s">
+      <c r="B10" s="16" t="s">
         <v>126</v>
       </c>
       <c r="C10" s="10">
@@ -2663,7 +2882,7 @@
       <c r="A11" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="B11" s="17" t="s">
+      <c r="B11" s="16" t="s">
         <v>126</v>
       </c>
       <c r="C11" s="10">
@@ -2676,7 +2895,7 @@
       <c r="A12" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="B12" s="17" t="s">
+      <c r="B12" s="16" t="s">
         <v>126</v>
       </c>
       <c r="C12" s="10">
@@ -2689,7 +2908,7 @@
       <c r="A13" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="B13" s="17" t="s">
+      <c r="B13" s="16" t="s">
         <v>126</v>
       </c>
       <c r="C13" s="10">
@@ -2702,7 +2921,7 @@
       <c r="A14" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="B14" s="17" t="s">
+      <c r="B14" s="16" t="s">
         <v>126</v>
       </c>
       <c r="C14" s="10">
@@ -2715,7 +2934,7 @@
       <c r="A15" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="B15" s="17" t="s">
+      <c r="B15" s="16" t="s">
         <v>126</v>
       </c>
       <c r="C15" s="10">
@@ -2728,7 +2947,7 @@
       <c r="A16" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="B16" s="17" t="s">
+      <c r="B16" s="16" t="s">
         <v>126</v>
       </c>
       <c r="C16" s="10">
@@ -2741,7 +2960,7 @@
       <c r="A17" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="B17" s="17" t="s">
+      <c r="B17" s="16" t="s">
         <v>126</v>
       </c>
       <c r="C17" s="10">
@@ -2754,7 +2973,7 @@
       <c r="A18" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="B18" s="17" t="s">
+      <c r="B18" s="16" t="s">
         <v>126</v>
       </c>
       <c r="C18" s="10">
@@ -2767,7 +2986,7 @@
       <c r="A19" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="B19" s="17" t="s">
+      <c r="B19" s="16" t="s">
         <v>127</v>
       </c>
       <c r="C19" s="10">
@@ -2780,7 +2999,7 @@
       <c r="A20" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="B20" s="17" t="s">
+      <c r="B20" s="16" t="s">
         <v>127</v>
       </c>
       <c r="C20" s="10">
@@ -2793,7 +3012,7 @@
       <c r="A21" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="B21" s="17" t="s">
+      <c r="B21" s="16" t="s">
         <v>127</v>
       </c>
       <c r="C21" s="10">
@@ -2806,7 +3025,7 @@
       <c r="A22" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="B22" s="17" t="s">
+      <c r="B22" s="16" t="s">
         <v>127</v>
       </c>
       <c r="C22" s="10">
@@ -2819,7 +3038,7 @@
       <c r="A23" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="B23" s="17" t="s">
+      <c r="B23" s="16" t="s">
         <v>127</v>
       </c>
       <c r="C23" s="10">
@@ -3327,4 +3546,2362 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9263046-FE36-46C5-AE2F-052E66BED452}">
+  <dimension ref="A1:E91"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="44" style="2" customWidth="1"/>
+    <col min="2" max="2" width="44" style="10" customWidth="1"/>
+    <col min="3" max="3" width="44" style="2" customWidth="1"/>
+    <col min="4" max="4" width="48.5703125" style="5" customWidth="1"/>
+    <col min="5" max="5" width="22" style="5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" s="1" customFormat="1" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="17" t="s">
+        <v>77</v>
+      </c>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+    </row>
+    <row r="2" spans="1:5" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="69" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="4">
+        <v>2</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="3"/>
+    </row>
+    <row r="5" spans="1:5" ht="69" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="C5" s="4"/>
+    </row>
+    <row r="6" spans="1:5" s="7" customFormat="1" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="12"/>
+      <c r="B6" s="12"/>
+      <c r="C6" s="8"/>
+      <c r="D6" s="6"/>
+      <c r="E6" s="6"/>
+    </row>
+    <row r="7" spans="1:5" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="D7" s="11" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="3.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="B8" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="D8" s="14" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B9" s="16" t="s">
+        <v>131</v>
+      </c>
+      <c r="C9" s="10">
+        <v>15</v>
+      </c>
+      <c r="D9" s="15" t="s">
+        <v>151</v>
+      </c>
+      <c r="E9" s="2"/>
+    </row>
+    <row r="10" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B10" s="16" t="s">
+        <v>132</v>
+      </c>
+      <c r="C10" s="10">
+        <v>15</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="E10" s="2"/>
+    </row>
+    <row r="11" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B11" s="16" t="s">
+        <v>86</v>
+      </c>
+      <c r="C11" s="10">
+        <v>15</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="E11" s="2"/>
+    </row>
+    <row r="12" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B12" s="16" t="s">
+        <v>133</v>
+      </c>
+      <c r="C12" s="10">
+        <v>15</v>
+      </c>
+      <c r="D12" s="15" t="s">
+        <v>153</v>
+      </c>
+      <c r="E12" s="2"/>
+    </row>
+    <row r="13" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B13" s="16" t="s">
+        <v>134</v>
+      </c>
+      <c r="C13" s="10">
+        <v>15</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="E13" s="2"/>
+    </row>
+    <row r="14" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B14" s="16" t="s">
+        <v>135</v>
+      </c>
+      <c r="C14" s="10">
+        <v>15</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="E14" s="2"/>
+    </row>
+    <row r="15" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B15" s="16" t="s">
+        <v>136</v>
+      </c>
+      <c r="C15" s="10">
+        <v>20</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="E15" s="2"/>
+    </row>
+    <row r="16" spans="1:5" s="9" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B16" s="16" t="s">
+        <v>137</v>
+      </c>
+      <c r="C16" s="10">
+        <v>15</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="E16" s="2"/>
+    </row>
+    <row r="17" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B17" s="16" t="s">
+        <v>138</v>
+      </c>
+      <c r="C17" s="10">
+        <v>20</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="E17" s="2"/>
+    </row>
+    <row r="18" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="B18" s="16" t="s">
+        <v>127</v>
+      </c>
+      <c r="C18" s="10">
+        <v>15</v>
+      </c>
+      <c r="D18" s="1"/>
+      <c r="E18" s="2"/>
+    </row>
+    <row r="19" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="B19" s="16" t="s">
+        <v>126</v>
+      </c>
+      <c r="C19" s="10">
+        <v>20</v>
+      </c>
+      <c r="D19" s="1"/>
+      <c r="E19" s="2"/>
+    </row>
+    <row r="20" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="B20" s="16" t="s">
+        <v>126</v>
+      </c>
+      <c r="C20" s="10">
+        <v>20</v>
+      </c>
+      <c r="D20" s="1"/>
+      <c r="E20" s="2"/>
+    </row>
+    <row r="21" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="B21" s="16" t="s">
+        <v>126</v>
+      </c>
+      <c r="C21" s="10">
+        <v>20</v>
+      </c>
+      <c r="D21" s="1"/>
+      <c r="E21" s="2"/>
+    </row>
+    <row r="22" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B22" s="16" t="s">
+        <v>126</v>
+      </c>
+      <c r="C22" s="10">
+        <v>15</v>
+      </c>
+      <c r="D22" s="1"/>
+      <c r="E22" s="2"/>
+    </row>
+    <row r="23" spans="1:5" s="9" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A23" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="B23" s="16" t="s">
+        <v>126</v>
+      </c>
+      <c r="C23" s="10">
+        <v>15</v>
+      </c>
+      <c r="D23" s="1"/>
+      <c r="E23" s="2"/>
+    </row>
+    <row r="24" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B24" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="C24" s="10">
+        <v>15</v>
+      </c>
+      <c r="D24" s="1"/>
+      <c r="E24" s="2"/>
+    </row>
+    <row r="25" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="B25" s="10" t="s">
+        <v>149</v>
+      </c>
+      <c r="C25" s="10">
+        <v>30</v>
+      </c>
+      <c r="D25" s="1"/>
+      <c r="E25" s="2"/>
+    </row>
+    <row r="26" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="B26" s="16" t="s">
+        <v>126</v>
+      </c>
+      <c r="C26" s="10">
+        <v>15</v>
+      </c>
+      <c r="D26" s="1"/>
+      <c r="E26" s="2"/>
+    </row>
+    <row r="27" spans="1:5" s="9" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A27" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="B27" s="10" t="s">
+        <v>150</v>
+      </c>
+      <c r="C27" s="10">
+        <v>15</v>
+      </c>
+      <c r="D27" s="1"/>
+      <c r="E27" s="2"/>
+    </row>
+    <row r="28" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="2"/>
+      <c r="B28" s="10"/>
+      <c r="C28" s="10"/>
+      <c r="D28" s="1"/>
+      <c r="E28" s="2"/>
+    </row>
+    <row r="29" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="2"/>
+      <c r="B29" s="10"/>
+      <c r="C29" s="10"/>
+      <c r="D29" s="1"/>
+      <c r="E29" s="2"/>
+    </row>
+    <row r="30" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="2"/>
+      <c r="B30" s="10"/>
+      <c r="C30" s="10"/>
+      <c r="D30" s="1"/>
+      <c r="E30" s="2"/>
+    </row>
+    <row r="31" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="2"/>
+      <c r="B31" s="10"/>
+      <c r="C31" s="10"/>
+      <c r="D31" s="1"/>
+      <c r="E31" s="2"/>
+    </row>
+    <row r="32" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="2"/>
+      <c r="B32" s="10"/>
+      <c r="C32" s="10"/>
+      <c r="D32" s="1"/>
+      <c r="E32" s="2"/>
+    </row>
+    <row r="33" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="2"/>
+      <c r="B33" s="10"/>
+      <c r="C33" s="10"/>
+      <c r="D33" s="1"/>
+      <c r="E33" s="2"/>
+    </row>
+    <row r="34" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="2"/>
+      <c r="B34" s="10"/>
+      <c r="C34" s="10"/>
+      <c r="D34" s="1"/>
+      <c r="E34" s="2"/>
+    </row>
+    <row r="35" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="2"/>
+      <c r="B35" s="10"/>
+      <c r="C35" s="10"/>
+      <c r="D35" s="1"/>
+      <c r="E35" s="2"/>
+    </row>
+    <row r="36" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="2"/>
+      <c r="B36" s="10"/>
+      <c r="C36" s="10"/>
+      <c r="D36" s="1"/>
+      <c r="E36" s="2"/>
+    </row>
+    <row r="37" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="2"/>
+      <c r="B37" s="10"/>
+      <c r="C37" s="10"/>
+      <c r="D37" s="1"/>
+      <c r="E37" s="2"/>
+    </row>
+    <row r="38" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="2"/>
+      <c r="B38" s="10"/>
+      <c r="C38" s="10"/>
+      <c r="D38" s="1"/>
+      <c r="E38" s="2"/>
+    </row>
+    <row r="39" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="2"/>
+      <c r="B39" s="10"/>
+      <c r="C39" s="10"/>
+      <c r="D39" s="5"/>
+      <c r="E39" s="2"/>
+    </row>
+    <row r="40" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="2"/>
+      <c r="B40" s="10"/>
+      <c r="C40" s="10"/>
+      <c r="D40" s="5"/>
+      <c r="E40" s="2"/>
+    </row>
+    <row r="41" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="2"/>
+      <c r="B41" s="10"/>
+      <c r="C41" s="10"/>
+      <c r="D41" s="5"/>
+      <c r="E41" s="2"/>
+    </row>
+    <row r="42" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="2"/>
+      <c r="B42" s="10"/>
+      <c r="C42" s="10"/>
+      <c r="D42" s="5"/>
+      <c r="E42" s="2"/>
+    </row>
+    <row r="43" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="2"/>
+      <c r="B43" s="10"/>
+      <c r="C43" s="10"/>
+      <c r="D43" s="5"/>
+      <c r="E43" s="2"/>
+    </row>
+    <row r="44" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="2"/>
+      <c r="B44" s="10"/>
+      <c r="C44" s="10"/>
+      <c r="D44" s="5"/>
+      <c r="E44" s="2"/>
+    </row>
+    <row r="45" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="2"/>
+      <c r="B45" s="10"/>
+      <c r="C45" s="10"/>
+      <c r="D45" s="5"/>
+      <c r="E45" s="2"/>
+    </row>
+    <row r="46" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="2"/>
+      <c r="B46" s="10"/>
+      <c r="C46" s="10"/>
+      <c r="D46" s="5"/>
+      <c r="E46" s="2"/>
+    </row>
+    <row r="47" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="2"/>
+      <c r="B47" s="10"/>
+      <c r="C47" s="10"/>
+      <c r="D47" s="5"/>
+      <c r="E47" s="2"/>
+    </row>
+    <row r="48" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="2"/>
+      <c r="B48" s="10"/>
+      <c r="C48" s="10"/>
+      <c r="D48" s="5"/>
+      <c r="E48" s="2"/>
+    </row>
+    <row r="49" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="2"/>
+      <c r="B49" s="10"/>
+      <c r="C49" s="10"/>
+      <c r="D49" s="5"/>
+      <c r="E49" s="2"/>
+    </row>
+    <row r="50" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="2"/>
+      <c r="B50" s="10"/>
+      <c r="C50" s="10"/>
+      <c r="D50" s="5"/>
+      <c r="E50" s="2"/>
+    </row>
+    <row r="51" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="2"/>
+      <c r="B51" s="10"/>
+      <c r="C51" s="10"/>
+      <c r="D51" s="5"/>
+      <c r="E51" s="2"/>
+    </row>
+    <row r="52" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A52" s="2"/>
+      <c r="B52" s="10"/>
+      <c r="C52" s="10"/>
+      <c r="D52" s="5"/>
+      <c r="E52" s="2"/>
+    </row>
+    <row r="53" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A53" s="2"/>
+      <c r="B53" s="10"/>
+      <c r="C53" s="10"/>
+      <c r="D53" s="5"/>
+      <c r="E53" s="2"/>
+    </row>
+    <row r="54" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A54" s="2"/>
+      <c r="B54" s="10"/>
+      <c r="C54" s="10"/>
+      <c r="D54" s="5"/>
+      <c r="E54" s="2"/>
+    </row>
+    <row r="55" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="2"/>
+      <c r="B55" s="10"/>
+      <c r="C55" s="10"/>
+      <c r="D55" s="5"/>
+      <c r="E55" s="2"/>
+    </row>
+    <row r="56" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A56" s="2"/>
+      <c r="B56" s="10"/>
+      <c r="C56" s="10"/>
+      <c r="D56" s="5"/>
+      <c r="E56" s="2"/>
+    </row>
+    <row r="57" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A57" s="2"/>
+      <c r="B57" s="10"/>
+      <c r="C57" s="10"/>
+      <c r="D57" s="5"/>
+      <c r="E57" s="2"/>
+    </row>
+    <row r="58" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A58" s="2"/>
+      <c r="B58" s="10"/>
+      <c r="C58" s="10"/>
+      <c r="D58" s="5"/>
+      <c r="E58" s="2"/>
+    </row>
+    <row r="59" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A59" s="2"/>
+      <c r="B59" s="10"/>
+      <c r="C59" s="10"/>
+      <c r="D59" s="5"/>
+      <c r="E59" s="2"/>
+    </row>
+    <row r="60" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A60" s="2"/>
+      <c r="B60" s="10"/>
+      <c r="C60" s="10"/>
+      <c r="D60" s="5"/>
+      <c r="E60" s="2"/>
+    </row>
+    <row r="61" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A61" s="2"/>
+      <c r="B61" s="10"/>
+      <c r="C61" s="10"/>
+      <c r="D61" s="5"/>
+      <c r="E61" s="2"/>
+    </row>
+    <row r="62" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A62" s="2"/>
+      <c r="B62" s="10"/>
+      <c r="C62" s="10"/>
+      <c r="D62" s="5"/>
+      <c r="E62" s="2"/>
+    </row>
+    <row r="63" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A63" s="2"/>
+      <c r="B63" s="10"/>
+      <c r="C63" s="10"/>
+      <c r="D63" s="5"/>
+      <c r="E63" s="2"/>
+    </row>
+    <row r="64" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A64" s="2"/>
+      <c r="B64" s="10"/>
+      <c r="C64" s="10"/>
+      <c r="D64" s="5"/>
+      <c r="E64" s="2"/>
+    </row>
+    <row r="65" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A65" s="2"/>
+      <c r="B65" s="10"/>
+      <c r="C65" s="10"/>
+      <c r="D65" s="5"/>
+      <c r="E65" s="2"/>
+    </row>
+    <row r="66" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A66" s="2"/>
+      <c r="B66" s="10"/>
+      <c r="C66" s="10"/>
+      <c r="D66" s="5"/>
+      <c r="E66" s="2"/>
+    </row>
+    <row r="67" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A67" s="2"/>
+      <c r="B67" s="10"/>
+      <c r="C67" s="10"/>
+      <c r="D67" s="5"/>
+      <c r="E67" s="2"/>
+    </row>
+    <row r="68" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A68" s="2"/>
+      <c r="B68" s="10"/>
+      <c r="C68" s="10"/>
+      <c r="D68" s="5"/>
+      <c r="E68" s="2"/>
+    </row>
+    <row r="69" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A69" s="2"/>
+      <c r="B69" s="10"/>
+      <c r="C69" s="10"/>
+      <c r="D69" s="5"/>
+      <c r="E69" s="2"/>
+    </row>
+    <row r="70" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A70" s="2"/>
+      <c r="B70" s="10"/>
+      <c r="C70" s="10"/>
+      <c r="D70" s="5"/>
+      <c r="E70" s="2"/>
+    </row>
+    <row r="71" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A71" s="2"/>
+      <c r="B71" s="10"/>
+      <c r="C71" s="10"/>
+      <c r="D71" s="5"/>
+      <c r="E71" s="2"/>
+    </row>
+    <row r="72" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A72" s="2"/>
+      <c r="B72" s="10"/>
+      <c r="C72" s="10"/>
+      <c r="D72" s="5"/>
+      <c r="E72" s="2"/>
+    </row>
+    <row r="73" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A73" s="2"/>
+      <c r="B73" s="10"/>
+      <c r="C73" s="10"/>
+      <c r="D73" s="5"/>
+      <c r="E73" s="2"/>
+    </row>
+    <row r="74" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A74" s="2"/>
+      <c r="B74" s="10"/>
+      <c r="C74" s="10"/>
+      <c r="D74" s="5"/>
+      <c r="E74" s="2"/>
+    </row>
+    <row r="75" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A75" s="2"/>
+      <c r="B75" s="10"/>
+      <c r="C75" s="10"/>
+      <c r="D75" s="5"/>
+      <c r="E75" s="2"/>
+    </row>
+    <row r="76" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A76" s="2"/>
+      <c r="B76" s="10"/>
+      <c r="C76" s="10"/>
+      <c r="D76" s="5"/>
+      <c r="E76" s="2"/>
+    </row>
+    <row r="77" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A77" s="2"/>
+      <c r="B77" s="10"/>
+      <c r="C77" s="10"/>
+      <c r="D77" s="5"/>
+      <c r="E77" s="2"/>
+    </row>
+    <row r="78" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A78" s="2"/>
+      <c r="B78" s="10"/>
+      <c r="C78" s="10"/>
+      <c r="D78" s="5"/>
+      <c r="E78" s="2"/>
+    </row>
+    <row r="79" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A79" s="2"/>
+      <c r="B79" s="10"/>
+      <c r="C79" s="10"/>
+      <c r="D79" s="5"/>
+      <c r="E79" s="2"/>
+    </row>
+    <row r="80" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A80" s="2"/>
+      <c r="B80" s="10"/>
+      <c r="C80" s="2"/>
+      <c r="D80" s="5"/>
+      <c r="E80" s="2"/>
+    </row>
+    <row r="81" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A81" s="2"/>
+      <c r="B81" s="10"/>
+      <c r="C81" s="2"/>
+      <c r="D81" s="5"/>
+      <c r="E81" s="2"/>
+    </row>
+    <row r="82" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A82" s="2"/>
+      <c r="B82" s="10"/>
+      <c r="C82" s="2"/>
+      <c r="D82" s="5"/>
+      <c r="E82" s="2"/>
+    </row>
+    <row r="83" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A83" s="2"/>
+      <c r="B83" s="10"/>
+      <c r="C83" s="2"/>
+      <c r="D83" s="5"/>
+      <c r="E83" s="2"/>
+    </row>
+    <row r="84" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A84" s="2"/>
+      <c r="B84" s="10"/>
+      <c r="C84" s="2"/>
+      <c r="D84" s="5"/>
+      <c r="E84" s="2"/>
+    </row>
+    <row r="85" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A85" s="2"/>
+      <c r="B85" s="10"/>
+      <c r="C85" s="2"/>
+      <c r="D85" s="5"/>
+      <c r="E85" s="2"/>
+    </row>
+    <row r="86" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A86" s="2"/>
+      <c r="B86" s="10"/>
+      <c r="C86" s="2"/>
+      <c r="D86" s="5"/>
+      <c r="E86" s="2"/>
+    </row>
+    <row r="87" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A87" s="2"/>
+      <c r="B87" s="10"/>
+      <c r="C87" s="2"/>
+      <c r="D87" s="5"/>
+      <c r="E87" s="2"/>
+    </row>
+    <row r="88" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A88" s="2"/>
+      <c r="B88" s="10"/>
+      <c r="C88" s="2"/>
+      <c r="D88" s="5"/>
+      <c r="E88" s="2"/>
+    </row>
+    <row r="89" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A89" s="2"/>
+      <c r="B89" s="10"/>
+      <c r="C89" s="2"/>
+      <c r="D89" s="5"/>
+      <c r="E89" s="2"/>
+    </row>
+    <row r="90" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A90" s="2"/>
+      <c r="B90" s="10"/>
+      <c r="C90" s="2"/>
+      <c r="D90" s="5"/>
+      <c r="E90" s="2"/>
+    </row>
+    <row r="91" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A91" s="2"/>
+      <c r="B91" s="10"/>
+      <c r="C91" s="2"/>
+      <c r="D91" s="5"/>
+      <c r="E91" s="2"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <dataValidations count="4">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C9:C249" xr:uid="{4A08B46B-060F-4B07-A887-3D578148E95E}">
+      <formula1>1</formula1>
+      <formula2>30</formula2>
+    </dataValidation>
+    <dataValidation type="textLength" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B3" xr:uid="{8BB62955-0962-4318-98D0-9762E7374531}">
+      <formula1>3</formula1>
+      <formula2>25</formula2>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A5" xr:uid="{0AA1F619-98FD-46E2-8C4B-4B09F6B8FFC2}">
+      <formula1>"English, Computer, Science, Math, Geography, History, General Knowledge, Social Studies, Life Skills"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A3" xr:uid="{020646C2-9FE4-4CD3-B61B-6958299D44F4}">
+      <formula1>"KG, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, Other"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="D12" r:id="rId1" xr:uid="{F2BDF28A-EEE3-412B-9045-F93536038E34}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16BE6E6A-CFE5-4EEB-AB25-4CDF6513BCB5}">
+  <dimension ref="A1:E83"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="44" style="2" customWidth="1"/>
+    <col min="2" max="2" width="44" style="10" customWidth="1"/>
+    <col min="3" max="3" width="44" style="2" customWidth="1"/>
+    <col min="4" max="4" width="48.5703125" style="5" customWidth="1"/>
+    <col min="5" max="5" width="22" style="5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" s="1" customFormat="1" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="17" t="s">
+        <v>77</v>
+      </c>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+    </row>
+    <row r="2" spans="1:5" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="69" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="3"/>
+    </row>
+    <row r="5" spans="1:5" ht="69" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="C5" s="4"/>
+    </row>
+    <row r="6" spans="1:5" s="7" customFormat="1" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="12"/>
+      <c r="B6" s="12"/>
+      <c r="C6" s="8"/>
+      <c r="D6" s="6"/>
+      <c r="E6" s="6"/>
+    </row>
+    <row r="7" spans="1:5" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="D7" s="11" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="3.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="B8" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="D8" s="14" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B9" s="16" t="s">
+        <v>131</v>
+      </c>
+      <c r="C9" s="10">
+        <v>20</v>
+      </c>
+      <c r="D9" s="15" t="s">
+        <v>151</v>
+      </c>
+      <c r="E9" s="2"/>
+    </row>
+    <row r="10" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B10" s="16" t="s">
+        <v>132</v>
+      </c>
+      <c r="C10" s="10">
+        <v>20</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="E10" s="2"/>
+    </row>
+    <row r="11" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B11" s="16" t="s">
+        <v>86</v>
+      </c>
+      <c r="C11" s="10">
+        <v>20</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="E11" s="2"/>
+    </row>
+    <row r="12" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B12" s="16" t="s">
+        <v>133</v>
+      </c>
+      <c r="C12" s="10">
+        <v>20</v>
+      </c>
+      <c r="D12" s="15" t="s">
+        <v>153</v>
+      </c>
+      <c r="E12" s="2"/>
+    </row>
+    <row r="13" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B13" s="16" t="s">
+        <v>134</v>
+      </c>
+      <c r="C13" s="10">
+        <v>20</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="E13" s="2"/>
+    </row>
+    <row r="14" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B14" s="16" t="s">
+        <v>135</v>
+      </c>
+      <c r="C14" s="10">
+        <v>20</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="E14" s="2"/>
+    </row>
+    <row r="15" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="B15" s="16" t="s">
+        <v>126</v>
+      </c>
+      <c r="C15" s="10">
+        <v>20</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="E15" s="2"/>
+    </row>
+    <row r="16" spans="1:5" s="9" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="B16" s="16" t="s">
+        <v>132</v>
+      </c>
+      <c r="C16" s="10">
+        <v>30</v>
+      </c>
+      <c r="D16" s="1"/>
+      <c r="E16" s="2"/>
+    </row>
+    <row r="17" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="B17" s="16" t="s">
+        <v>133</v>
+      </c>
+      <c r="C17" s="10">
+        <v>30</v>
+      </c>
+      <c r="D17" s="1"/>
+      <c r="E17" s="2"/>
+    </row>
+    <row r="18" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="B18" s="16" t="s">
+        <v>86</v>
+      </c>
+      <c r="C18" s="10">
+        <v>30</v>
+      </c>
+      <c r="D18" s="1"/>
+      <c r="E18" s="2"/>
+    </row>
+    <row r="19" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="B19" s="16" t="s">
+        <v>131</v>
+      </c>
+      <c r="C19" s="10">
+        <v>30</v>
+      </c>
+      <c r="D19" s="1"/>
+      <c r="E19" s="2"/>
+    </row>
+    <row r="20" spans="1:5" s="9" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="B20" s="16" t="s">
+        <v>135</v>
+      </c>
+      <c r="C20" s="10">
+        <v>30</v>
+      </c>
+      <c r="D20" s="1"/>
+      <c r="E20" s="2"/>
+    </row>
+    <row r="21" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="B21" s="16" t="s">
+        <v>134</v>
+      </c>
+      <c r="C21" s="10">
+        <v>30</v>
+      </c>
+      <c r="D21" s="1"/>
+      <c r="E21" s="2"/>
+    </row>
+    <row r="22" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="2"/>
+      <c r="B22" s="10"/>
+      <c r="C22" s="10"/>
+      <c r="D22" s="1"/>
+      <c r="E22" s="2"/>
+    </row>
+    <row r="23" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="2"/>
+      <c r="B23" s="10"/>
+      <c r="C23" s="10"/>
+      <c r="D23" s="1"/>
+      <c r="E23" s="2"/>
+    </row>
+    <row r="24" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="2"/>
+      <c r="B24" s="10"/>
+      <c r="C24" s="10"/>
+      <c r="D24" s="1"/>
+      <c r="E24" s="2"/>
+    </row>
+    <row r="25" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="2"/>
+      <c r="B25" s="10"/>
+      <c r="C25" s="10"/>
+      <c r="D25" s="1"/>
+      <c r="E25" s="2"/>
+    </row>
+    <row r="26" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="2"/>
+      <c r="B26" s="10"/>
+      <c r="C26" s="10"/>
+      <c r="D26" s="1"/>
+      <c r="E26" s="2"/>
+    </row>
+    <row r="27" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="2"/>
+      <c r="B27" s="10"/>
+      <c r="C27" s="10"/>
+      <c r="D27" s="1"/>
+      <c r="E27" s="2"/>
+    </row>
+    <row r="28" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="2"/>
+      <c r="B28" s="10"/>
+      <c r="C28" s="10"/>
+      <c r="D28" s="1"/>
+      <c r="E28" s="2"/>
+    </row>
+    <row r="29" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="2"/>
+      <c r="B29" s="10"/>
+      <c r="C29" s="10"/>
+      <c r="D29" s="1"/>
+      <c r="E29" s="2"/>
+    </row>
+    <row r="30" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="2"/>
+      <c r="B30" s="10"/>
+      <c r="C30" s="10"/>
+      <c r="D30" s="1"/>
+      <c r="E30" s="2"/>
+    </row>
+    <row r="31" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="2"/>
+      <c r="B31" s="10"/>
+      <c r="C31" s="10"/>
+      <c r="D31" s="5"/>
+      <c r="E31" s="2"/>
+    </row>
+    <row r="32" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="2"/>
+      <c r="B32" s="10"/>
+      <c r="C32" s="10"/>
+      <c r="D32" s="5"/>
+      <c r="E32" s="2"/>
+    </row>
+    <row r="33" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="2"/>
+      <c r="B33" s="10"/>
+      <c r="C33" s="10"/>
+      <c r="D33" s="5"/>
+      <c r="E33" s="2"/>
+    </row>
+    <row r="34" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="2"/>
+      <c r="B34" s="10"/>
+      <c r="C34" s="10"/>
+      <c r="D34" s="5"/>
+      <c r="E34" s="2"/>
+    </row>
+    <row r="35" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="2"/>
+      <c r="B35" s="10"/>
+      <c r="C35" s="10"/>
+      <c r="D35" s="5"/>
+      <c r="E35" s="2"/>
+    </row>
+    <row r="36" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="2"/>
+      <c r="B36" s="10"/>
+      <c r="C36" s="10"/>
+      <c r="D36" s="5"/>
+      <c r="E36" s="2"/>
+    </row>
+    <row r="37" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="2"/>
+      <c r="B37" s="10"/>
+      <c r="C37" s="10"/>
+      <c r="D37" s="5"/>
+      <c r="E37" s="2"/>
+    </row>
+    <row r="38" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="2"/>
+      <c r="B38" s="10"/>
+      <c r="C38" s="10"/>
+      <c r="D38" s="5"/>
+      <c r="E38" s="2"/>
+    </row>
+    <row r="39" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="2"/>
+      <c r="B39" s="10"/>
+      <c r="C39" s="10"/>
+      <c r="D39" s="5"/>
+      <c r="E39" s="2"/>
+    </row>
+    <row r="40" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="2"/>
+      <c r="B40" s="10"/>
+      <c r="C40" s="10"/>
+      <c r="D40" s="5"/>
+      <c r="E40" s="2"/>
+    </row>
+    <row r="41" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="2"/>
+      <c r="B41" s="10"/>
+      <c r="C41" s="10"/>
+      <c r="D41" s="5"/>
+      <c r="E41" s="2"/>
+    </row>
+    <row r="42" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="2"/>
+      <c r="B42" s="10"/>
+      <c r="C42" s="10"/>
+      <c r="D42" s="5"/>
+      <c r="E42" s="2"/>
+    </row>
+    <row r="43" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="2"/>
+      <c r="B43" s="10"/>
+      <c r="C43" s="10"/>
+      <c r="D43" s="5"/>
+      <c r="E43" s="2"/>
+    </row>
+    <row r="44" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="2"/>
+      <c r="B44" s="10"/>
+      <c r="C44" s="10"/>
+      <c r="D44" s="5"/>
+      <c r="E44" s="2"/>
+    </row>
+    <row r="45" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="2"/>
+      <c r="B45" s="10"/>
+      <c r="C45" s="10"/>
+      <c r="D45" s="5"/>
+      <c r="E45" s="2"/>
+    </row>
+    <row r="46" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="2"/>
+      <c r="B46" s="10"/>
+      <c r="C46" s="10"/>
+      <c r="D46" s="5"/>
+      <c r="E46" s="2"/>
+    </row>
+    <row r="47" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="2"/>
+      <c r="B47" s="10"/>
+      <c r="C47" s="10"/>
+      <c r="D47" s="5"/>
+      <c r="E47" s="2"/>
+    </row>
+    <row r="48" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="2"/>
+      <c r="B48" s="10"/>
+      <c r="C48" s="10"/>
+      <c r="D48" s="5"/>
+      <c r="E48" s="2"/>
+    </row>
+    <row r="49" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="2"/>
+      <c r="B49" s="10"/>
+      <c r="C49" s="10"/>
+      <c r="D49" s="5"/>
+      <c r="E49" s="2"/>
+    </row>
+    <row r="50" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="2"/>
+      <c r="B50" s="10"/>
+      <c r="C50" s="10"/>
+      <c r="D50" s="5"/>
+      <c r="E50" s="2"/>
+    </row>
+    <row r="51" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="2"/>
+      <c r="B51" s="10"/>
+      <c r="C51" s="10"/>
+      <c r="D51" s="5"/>
+      <c r="E51" s="2"/>
+    </row>
+    <row r="52" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A52" s="2"/>
+      <c r="B52" s="10"/>
+      <c r="C52" s="10"/>
+      <c r="D52" s="5"/>
+      <c r="E52" s="2"/>
+    </row>
+    <row r="53" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A53" s="2"/>
+      <c r="B53" s="10"/>
+      <c r="C53" s="10"/>
+      <c r="D53" s="5"/>
+      <c r="E53" s="2"/>
+    </row>
+    <row r="54" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A54" s="2"/>
+      <c r="B54" s="10"/>
+      <c r="C54" s="10"/>
+      <c r="D54" s="5"/>
+      <c r="E54" s="2"/>
+    </row>
+    <row r="55" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="2"/>
+      <c r="B55" s="10"/>
+      <c r="C55" s="10"/>
+      <c r="D55" s="5"/>
+      <c r="E55" s="2"/>
+    </row>
+    <row r="56" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A56" s="2"/>
+      <c r="B56" s="10"/>
+      <c r="C56" s="10"/>
+      <c r="D56" s="5"/>
+      <c r="E56" s="2"/>
+    </row>
+    <row r="57" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A57" s="2"/>
+      <c r="B57" s="10"/>
+      <c r="C57" s="10"/>
+      <c r="D57" s="5"/>
+      <c r="E57" s="2"/>
+    </row>
+    <row r="58" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A58" s="2"/>
+      <c r="B58" s="10"/>
+      <c r="C58" s="10"/>
+      <c r="D58" s="5"/>
+      <c r="E58" s="2"/>
+    </row>
+    <row r="59" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A59" s="2"/>
+      <c r="B59" s="10"/>
+      <c r="C59" s="10"/>
+      <c r="D59" s="5"/>
+      <c r="E59" s="2"/>
+    </row>
+    <row r="60" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A60" s="2"/>
+      <c r="B60" s="10"/>
+      <c r="C60" s="10"/>
+      <c r="D60" s="5"/>
+      <c r="E60" s="2"/>
+    </row>
+    <row r="61" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A61" s="2"/>
+      <c r="B61" s="10"/>
+      <c r="C61" s="10"/>
+      <c r="D61" s="5"/>
+      <c r="E61" s="2"/>
+    </row>
+    <row r="62" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A62" s="2"/>
+      <c r="B62" s="10"/>
+      <c r="C62" s="10"/>
+      <c r="D62" s="5"/>
+      <c r="E62" s="2"/>
+    </row>
+    <row r="63" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A63" s="2"/>
+      <c r="B63" s="10"/>
+      <c r="C63" s="10"/>
+      <c r="D63" s="5"/>
+      <c r="E63" s="2"/>
+    </row>
+    <row r="64" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A64" s="2"/>
+      <c r="B64" s="10"/>
+      <c r="C64" s="10"/>
+      <c r="D64" s="5"/>
+      <c r="E64" s="2"/>
+    </row>
+    <row r="65" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A65" s="2"/>
+      <c r="B65" s="10"/>
+      <c r="C65" s="10"/>
+      <c r="D65" s="5"/>
+      <c r="E65" s="2"/>
+    </row>
+    <row r="66" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A66" s="2"/>
+      <c r="B66" s="10"/>
+      <c r="C66" s="10"/>
+      <c r="D66" s="5"/>
+      <c r="E66" s="2"/>
+    </row>
+    <row r="67" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A67" s="2"/>
+      <c r="B67" s="10"/>
+      <c r="C67" s="10"/>
+      <c r="D67" s="5"/>
+      <c r="E67" s="2"/>
+    </row>
+    <row r="68" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A68" s="2"/>
+      <c r="B68" s="10"/>
+      <c r="C68" s="10"/>
+      <c r="D68" s="5"/>
+      <c r="E68" s="2"/>
+    </row>
+    <row r="69" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A69" s="2"/>
+      <c r="B69" s="10"/>
+      <c r="C69" s="10"/>
+      <c r="D69" s="5"/>
+      <c r="E69" s="2"/>
+    </row>
+    <row r="70" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A70" s="2"/>
+      <c r="B70" s="10"/>
+      <c r="C70" s="10"/>
+      <c r="D70" s="5"/>
+      <c r="E70" s="2"/>
+    </row>
+    <row r="71" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A71" s="2"/>
+      <c r="B71" s="10"/>
+      <c r="C71" s="10"/>
+      <c r="D71" s="5"/>
+      <c r="E71" s="2"/>
+    </row>
+    <row r="72" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A72" s="2"/>
+      <c r="B72" s="10"/>
+      <c r="C72" s="2"/>
+      <c r="D72" s="5"/>
+      <c r="E72" s="2"/>
+    </row>
+    <row r="73" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A73" s="2"/>
+      <c r="B73" s="10"/>
+      <c r="C73" s="2"/>
+      <c r="D73" s="5"/>
+      <c r="E73" s="2"/>
+    </row>
+    <row r="74" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A74" s="2"/>
+      <c r="B74" s="10"/>
+      <c r="C74" s="2"/>
+      <c r="D74" s="5"/>
+      <c r="E74" s="2"/>
+    </row>
+    <row r="75" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A75" s="2"/>
+      <c r="B75" s="10"/>
+      <c r="C75" s="2"/>
+      <c r="D75" s="5"/>
+      <c r="E75" s="2"/>
+    </row>
+    <row r="76" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A76" s="2"/>
+      <c r="B76" s="10"/>
+      <c r="C76" s="2"/>
+      <c r="D76" s="5"/>
+      <c r="E76" s="2"/>
+    </row>
+    <row r="77" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A77" s="2"/>
+      <c r="B77" s="10"/>
+      <c r="C77" s="2"/>
+      <c r="D77" s="5"/>
+      <c r="E77" s="2"/>
+    </row>
+    <row r="78" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A78" s="2"/>
+      <c r="B78" s="10"/>
+      <c r="C78" s="2"/>
+      <c r="D78" s="5"/>
+      <c r="E78" s="2"/>
+    </row>
+    <row r="79" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A79" s="2"/>
+      <c r="B79" s="10"/>
+      <c r="C79" s="2"/>
+      <c r="D79" s="5"/>
+      <c r="E79" s="2"/>
+    </row>
+    <row r="80" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A80" s="2"/>
+      <c r="B80" s="10"/>
+      <c r="C80" s="2"/>
+      <c r="D80" s="5"/>
+      <c r="E80" s="2"/>
+    </row>
+    <row r="81" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A81" s="2"/>
+      <c r="B81" s="10"/>
+      <c r="C81" s="2"/>
+      <c r="D81" s="5"/>
+      <c r="E81" s="2"/>
+    </row>
+    <row r="82" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A82" s="2"/>
+      <c r="B82" s="10"/>
+      <c r="C82" s="2"/>
+      <c r="D82" s="5"/>
+      <c r="E82" s="2"/>
+    </row>
+    <row r="83" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A83" s="2"/>
+      <c r="B83" s="10"/>
+      <c r="C83" s="2"/>
+      <c r="D83" s="5"/>
+      <c r="E83" s="2"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <dataValidations count="4">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A3" xr:uid="{B198EC55-45BB-4B2C-9D68-49307776E0AE}">
+      <formula1>"KG, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, Other"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A5" xr:uid="{AF9C42EB-73BF-4C6E-BAFC-E72288147896}">
+      <formula1>"English, Computer, Science, Math, Geography, History, General Knowledge, Social Studies, Life Skills"</formula1>
+    </dataValidation>
+    <dataValidation type="textLength" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B3" xr:uid="{1A4BE707-90F7-4164-AB55-9ACF4DFE2ACE}">
+      <formula1>3</formula1>
+      <formula2>25</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C9:C241" xr:uid="{298E909D-7FE2-479E-84CA-E9B9CFC6CFE9}">
+      <formula1>1</formula1>
+      <formula2>30</formula2>
+    </dataValidation>
+  </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="D12" r:id="rId1" xr:uid="{B6C1CABB-A700-440B-8F3A-04FBCE1AB930}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF5EDB16-6A22-405A-8C30-5681553FE3DB}">
+  <dimension ref="A1:E91"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="44" style="2" customWidth="1"/>
+    <col min="2" max="2" width="44" style="10" customWidth="1"/>
+    <col min="3" max="3" width="44" style="2" customWidth="1"/>
+    <col min="4" max="4" width="48.5703125" style="5" customWidth="1"/>
+    <col min="5" max="5" width="22" style="5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" s="1" customFormat="1" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="17" t="s">
+        <v>77</v>
+      </c>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+    </row>
+    <row r="2" spans="1:5" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="69" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="4">
+        <v>5</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="3"/>
+    </row>
+    <row r="5" spans="1:5" ht="69" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="C5" s="4"/>
+    </row>
+    <row r="6" spans="1:5" s="7" customFormat="1" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="12"/>
+      <c r="B6" s="12"/>
+      <c r="C6" s="8"/>
+      <c r="D6" s="6"/>
+      <c r="E6" s="6"/>
+    </row>
+    <row r="7" spans="1:5" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="D7" s="11" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="3.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="B8" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="D8" s="14" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="B9" s="16" t="s">
+        <v>199</v>
+      </c>
+      <c r="C9" s="10">
+        <v>15</v>
+      </c>
+      <c r="D9" s="15"/>
+      <c r="E9" s="2"/>
+    </row>
+    <row r="10" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="B10" s="16" t="s">
+        <v>187</v>
+      </c>
+      <c r="C10" s="10">
+        <v>15</v>
+      </c>
+      <c r="D10" s="1"/>
+      <c r="E10" s="2"/>
+    </row>
+    <row r="11" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="B11" s="16" t="s">
+        <v>188</v>
+      </c>
+      <c r="C11" s="10">
+        <v>15</v>
+      </c>
+      <c r="D11" s="1"/>
+      <c r="E11" s="2"/>
+    </row>
+    <row r="12" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="B12" s="16" t="s">
+        <v>189</v>
+      </c>
+      <c r="C12" s="10">
+        <v>15</v>
+      </c>
+      <c r="D12" s="1"/>
+      <c r="E12" s="2"/>
+    </row>
+    <row r="13" spans="1:5" s="9" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="B13" s="16" t="s">
+        <v>190</v>
+      </c>
+      <c r="C13" s="10">
+        <v>20</v>
+      </c>
+      <c r="D13" s="1"/>
+      <c r="E13" s="2"/>
+    </row>
+    <row r="14" spans="1:5" s="9" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="B14" s="16" t="s">
+        <v>191</v>
+      </c>
+      <c r="C14" s="10">
+        <v>20</v>
+      </c>
+      <c r="D14" s="1"/>
+      <c r="E14" s="2"/>
+    </row>
+    <row r="15" spans="1:5" s="9" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="B15" s="16" t="s">
+        <v>192</v>
+      </c>
+      <c r="C15" s="10">
+        <v>20</v>
+      </c>
+      <c r="D15" s="1"/>
+      <c r="E15" s="2"/>
+    </row>
+    <row r="16" spans="1:5" s="9" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="B16" s="16" t="s">
+        <v>193</v>
+      </c>
+      <c r="C16" s="10">
+        <v>20</v>
+      </c>
+      <c r="D16" s="1"/>
+      <c r="E16" s="2"/>
+    </row>
+    <row r="17" spans="1:5" s="9" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="B17" s="16" t="s">
+        <v>194</v>
+      </c>
+      <c r="C17" s="10">
+        <v>30</v>
+      </c>
+      <c r="D17" s="1"/>
+      <c r="E17" s="2"/>
+    </row>
+    <row r="18" spans="1:5" s="9" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="B18" s="16" t="s">
+        <v>195</v>
+      </c>
+      <c r="C18" s="10">
+        <v>15</v>
+      </c>
+      <c r="D18" s="1"/>
+      <c r="E18" s="2"/>
+    </row>
+    <row r="19" spans="1:5" s="9" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="B19" s="16" t="s">
+        <v>196</v>
+      </c>
+      <c r="C19" s="10">
+        <v>15</v>
+      </c>
+      <c r="D19" s="1"/>
+      <c r="E19" s="2"/>
+    </row>
+    <row r="20" spans="1:5" s="9" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="B20" s="16" t="s">
+        <v>197</v>
+      </c>
+      <c r="C20" s="10">
+        <v>15</v>
+      </c>
+      <c r="D20" s="1"/>
+      <c r="E20" s="2"/>
+    </row>
+    <row r="21" spans="1:5" s="9" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="B21" s="16" t="s">
+        <v>194</v>
+      </c>
+      <c r="C21" s="10">
+        <v>15</v>
+      </c>
+      <c r="D21" s="1"/>
+      <c r="E21" s="2"/>
+    </row>
+    <row r="22" spans="1:5" s="9" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A22" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="B22" s="16" t="s">
+        <v>198</v>
+      </c>
+      <c r="C22" s="10">
+        <v>15</v>
+      </c>
+      <c r="D22" s="1"/>
+      <c r="E22" s="2"/>
+    </row>
+    <row r="23" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="2"/>
+      <c r="B23" s="16"/>
+      <c r="C23" s="10"/>
+      <c r="D23" s="1"/>
+      <c r="E23" s="2"/>
+    </row>
+    <row r="24" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="2"/>
+      <c r="B24" s="10"/>
+      <c r="C24" s="10"/>
+      <c r="D24" s="1"/>
+      <c r="E24" s="2"/>
+    </row>
+    <row r="25" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="2"/>
+      <c r="B25" s="10"/>
+      <c r="C25" s="10"/>
+      <c r="D25" s="1"/>
+      <c r="E25" s="2"/>
+    </row>
+    <row r="26" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="2"/>
+      <c r="B26" s="10"/>
+      <c r="C26" s="10"/>
+      <c r="D26" s="1"/>
+      <c r="E26" s="2"/>
+    </row>
+    <row r="27" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="2"/>
+      <c r="B27" s="10"/>
+      <c r="C27" s="10"/>
+      <c r="D27" s="1"/>
+      <c r="E27" s="2"/>
+    </row>
+    <row r="28" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="2"/>
+      <c r="B28" s="10"/>
+      <c r="C28" s="10"/>
+      <c r="D28" s="1"/>
+      <c r="E28" s="2"/>
+    </row>
+    <row r="29" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="2"/>
+      <c r="B29" s="10"/>
+      <c r="C29" s="10"/>
+      <c r="D29" s="1"/>
+      <c r="E29" s="2"/>
+    </row>
+    <row r="30" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="2"/>
+      <c r="B30" s="10"/>
+      <c r="C30" s="10"/>
+      <c r="D30" s="1"/>
+      <c r="E30" s="2"/>
+    </row>
+    <row r="31" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="2"/>
+      <c r="B31" s="10"/>
+      <c r="C31" s="10"/>
+      <c r="D31" s="1"/>
+      <c r="E31" s="2"/>
+    </row>
+    <row r="32" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="2"/>
+      <c r="B32" s="10"/>
+      <c r="C32" s="10"/>
+      <c r="D32" s="1"/>
+      <c r="E32" s="2"/>
+    </row>
+    <row r="33" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="2"/>
+      <c r="B33" s="10"/>
+      <c r="C33" s="10"/>
+      <c r="D33" s="1"/>
+      <c r="E33" s="2"/>
+    </row>
+    <row r="34" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="2"/>
+      <c r="B34" s="10"/>
+      <c r="C34" s="10"/>
+      <c r="D34" s="1"/>
+      <c r="E34" s="2"/>
+    </row>
+    <row r="35" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="2"/>
+      <c r="B35" s="10"/>
+      <c r="C35" s="10"/>
+      <c r="D35" s="1"/>
+      <c r="E35" s="2"/>
+    </row>
+    <row r="36" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="2"/>
+      <c r="B36" s="10"/>
+      <c r="C36" s="10"/>
+      <c r="D36" s="1"/>
+      <c r="E36" s="2"/>
+    </row>
+    <row r="37" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="2"/>
+      <c r="B37" s="10"/>
+      <c r="C37" s="10"/>
+      <c r="D37" s="1"/>
+      <c r="E37" s="2"/>
+    </row>
+    <row r="38" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="2"/>
+      <c r="B38" s="10"/>
+      <c r="C38" s="10"/>
+      <c r="D38" s="1"/>
+      <c r="E38" s="2"/>
+    </row>
+    <row r="39" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="2"/>
+      <c r="B39" s="10"/>
+      <c r="C39" s="10"/>
+      <c r="D39" s="5"/>
+      <c r="E39" s="2"/>
+    </row>
+    <row r="40" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="2"/>
+      <c r="B40" s="10"/>
+      <c r="C40" s="10"/>
+      <c r="D40" s="5"/>
+      <c r="E40" s="2"/>
+    </row>
+    <row r="41" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="2"/>
+      <c r="B41" s="10"/>
+      <c r="C41" s="10"/>
+      <c r="D41" s="5"/>
+      <c r="E41" s="2"/>
+    </row>
+    <row r="42" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="2"/>
+      <c r="B42" s="10"/>
+      <c r="C42" s="10"/>
+      <c r="D42" s="5"/>
+      <c r="E42" s="2"/>
+    </row>
+    <row r="43" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="2"/>
+      <c r="B43" s="10"/>
+      <c r="C43" s="10"/>
+      <c r="D43" s="5"/>
+      <c r="E43" s="2"/>
+    </row>
+    <row r="44" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="2"/>
+      <c r="B44" s="10"/>
+      <c r="C44" s="10"/>
+      <c r="D44" s="5"/>
+      <c r="E44" s="2"/>
+    </row>
+    <row r="45" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="2"/>
+      <c r="B45" s="10"/>
+      <c r="C45" s="10"/>
+      <c r="D45" s="5"/>
+      <c r="E45" s="2"/>
+    </row>
+    <row r="46" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="2"/>
+      <c r="B46" s="10"/>
+      <c r="C46" s="10"/>
+      <c r="D46" s="5"/>
+      <c r="E46" s="2"/>
+    </row>
+    <row r="47" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="2"/>
+      <c r="B47" s="10"/>
+      <c r="C47" s="10"/>
+      <c r="D47" s="5"/>
+      <c r="E47" s="2"/>
+    </row>
+    <row r="48" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="2"/>
+      <c r="B48" s="10"/>
+      <c r="C48" s="10"/>
+      <c r="D48" s="5"/>
+      <c r="E48" s="2"/>
+    </row>
+    <row r="49" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="2"/>
+      <c r="B49" s="10"/>
+      <c r="C49" s="10"/>
+      <c r="D49" s="5"/>
+      <c r="E49" s="2"/>
+    </row>
+    <row r="50" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="2"/>
+      <c r="B50" s="10"/>
+      <c r="C50" s="10"/>
+      <c r="D50" s="5"/>
+      <c r="E50" s="2"/>
+    </row>
+    <row r="51" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="2"/>
+      <c r="B51" s="10"/>
+      <c r="C51" s="10"/>
+      <c r="D51" s="5"/>
+      <c r="E51" s="2"/>
+    </row>
+    <row r="52" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A52" s="2"/>
+      <c r="B52" s="10"/>
+      <c r="C52" s="10"/>
+      <c r="D52" s="5"/>
+      <c r="E52" s="2"/>
+    </row>
+    <row r="53" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A53" s="2"/>
+      <c r="B53" s="10"/>
+      <c r="C53" s="10"/>
+      <c r="D53" s="5"/>
+      <c r="E53" s="2"/>
+    </row>
+    <row r="54" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A54" s="2"/>
+      <c r="B54" s="10"/>
+      <c r="C54" s="10"/>
+      <c r="D54" s="5"/>
+      <c r="E54" s="2"/>
+    </row>
+    <row r="55" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="2"/>
+      <c r="B55" s="10"/>
+      <c r="C55" s="10"/>
+      <c r="D55" s="5"/>
+      <c r="E55" s="2"/>
+    </row>
+    <row r="56" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A56" s="2"/>
+      <c r="B56" s="10"/>
+      <c r="C56" s="10"/>
+      <c r="D56" s="5"/>
+      <c r="E56" s="2"/>
+    </row>
+    <row r="57" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A57" s="2"/>
+      <c r="B57" s="10"/>
+      <c r="C57" s="10"/>
+      <c r="D57" s="5"/>
+      <c r="E57" s="2"/>
+    </row>
+    <row r="58" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A58" s="2"/>
+      <c r="B58" s="10"/>
+      <c r="C58" s="10"/>
+      <c r="D58" s="5"/>
+      <c r="E58" s="2"/>
+    </row>
+    <row r="59" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A59" s="2"/>
+      <c r="B59" s="10"/>
+      <c r="C59" s="10"/>
+      <c r="D59" s="5"/>
+      <c r="E59" s="2"/>
+    </row>
+    <row r="60" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A60" s="2"/>
+      <c r="B60" s="10"/>
+      <c r="C60" s="10"/>
+      <c r="D60" s="5"/>
+      <c r="E60" s="2"/>
+    </row>
+    <row r="61" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A61" s="2"/>
+      <c r="B61" s="10"/>
+      <c r="C61" s="10"/>
+      <c r="D61" s="5"/>
+      <c r="E61" s="2"/>
+    </row>
+    <row r="62" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A62" s="2"/>
+      <c r="B62" s="10"/>
+      <c r="C62" s="10"/>
+      <c r="D62" s="5"/>
+      <c r="E62" s="2"/>
+    </row>
+    <row r="63" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A63" s="2"/>
+      <c r="B63" s="10"/>
+      <c r="C63" s="10"/>
+      <c r="D63" s="5"/>
+      <c r="E63" s="2"/>
+    </row>
+    <row r="64" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A64" s="2"/>
+      <c r="B64" s="10"/>
+      <c r="C64" s="10"/>
+      <c r="D64" s="5"/>
+      <c r="E64" s="2"/>
+    </row>
+    <row r="65" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A65" s="2"/>
+      <c r="B65" s="10"/>
+      <c r="C65" s="10"/>
+      <c r="D65" s="5"/>
+      <c r="E65" s="2"/>
+    </row>
+    <row r="66" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A66" s="2"/>
+      <c r="B66" s="10"/>
+      <c r="C66" s="10"/>
+      <c r="D66" s="5"/>
+      <c r="E66" s="2"/>
+    </row>
+    <row r="67" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A67" s="2"/>
+      <c r="B67" s="10"/>
+      <c r="C67" s="10"/>
+      <c r="D67" s="5"/>
+      <c r="E67" s="2"/>
+    </row>
+    <row r="68" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A68" s="2"/>
+      <c r="B68" s="10"/>
+      <c r="C68" s="10"/>
+      <c r="D68" s="5"/>
+      <c r="E68" s="2"/>
+    </row>
+    <row r="69" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A69" s="2"/>
+      <c r="B69" s="10"/>
+      <c r="C69" s="10"/>
+      <c r="D69" s="5"/>
+      <c r="E69" s="2"/>
+    </row>
+    <row r="70" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A70" s="2"/>
+      <c r="B70" s="10"/>
+      <c r="C70" s="10"/>
+      <c r="D70" s="5"/>
+      <c r="E70" s="2"/>
+    </row>
+    <row r="71" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A71" s="2"/>
+      <c r="B71" s="10"/>
+      <c r="C71" s="10"/>
+      <c r="D71" s="5"/>
+      <c r="E71" s="2"/>
+    </row>
+    <row r="72" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A72" s="2"/>
+      <c r="B72" s="10"/>
+      <c r="C72" s="10"/>
+      <c r="D72" s="5"/>
+      <c r="E72" s="2"/>
+    </row>
+    <row r="73" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A73" s="2"/>
+      <c r="B73" s="10"/>
+      <c r="C73" s="10"/>
+      <c r="D73" s="5"/>
+      <c r="E73" s="2"/>
+    </row>
+    <row r="74" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A74" s="2"/>
+      <c r="B74" s="10"/>
+      <c r="C74" s="10"/>
+      <c r="D74" s="5"/>
+      <c r="E74" s="2"/>
+    </row>
+    <row r="75" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A75" s="2"/>
+      <c r="B75" s="10"/>
+      <c r="C75" s="10"/>
+      <c r="D75" s="5"/>
+      <c r="E75" s="2"/>
+    </row>
+    <row r="76" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A76" s="2"/>
+      <c r="B76" s="10"/>
+      <c r="C76" s="10"/>
+      <c r="D76" s="5"/>
+      <c r="E76" s="2"/>
+    </row>
+    <row r="77" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A77" s="2"/>
+      <c r="B77" s="10"/>
+      <c r="C77" s="10"/>
+      <c r="D77" s="5"/>
+      <c r="E77" s="2"/>
+    </row>
+    <row r="78" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A78" s="2"/>
+      <c r="B78" s="10"/>
+      <c r="C78" s="10"/>
+      <c r="D78" s="5"/>
+      <c r="E78" s="2"/>
+    </row>
+    <row r="79" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A79" s="2"/>
+      <c r="B79" s="10"/>
+      <c r="C79" s="10"/>
+      <c r="D79" s="5"/>
+      <c r="E79" s="2"/>
+    </row>
+    <row r="80" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A80" s="2"/>
+      <c r="B80" s="10"/>
+      <c r="C80" s="2"/>
+      <c r="D80" s="5"/>
+      <c r="E80" s="2"/>
+    </row>
+    <row r="81" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A81" s="2"/>
+      <c r="B81" s="10"/>
+      <c r="C81" s="2"/>
+      <c r="D81" s="5"/>
+      <c r="E81" s="2"/>
+    </row>
+    <row r="82" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A82" s="2"/>
+      <c r="B82" s="10"/>
+      <c r="C82" s="2"/>
+      <c r="D82" s="5"/>
+      <c r="E82" s="2"/>
+    </row>
+    <row r="83" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A83" s="2"/>
+      <c r="B83" s="10"/>
+      <c r="C83" s="2"/>
+      <c r="D83" s="5"/>
+      <c r="E83" s="2"/>
+    </row>
+    <row r="84" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A84" s="2"/>
+      <c r="B84" s="10"/>
+      <c r="C84" s="2"/>
+      <c r="D84" s="5"/>
+      <c r="E84" s="2"/>
+    </row>
+    <row r="85" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A85" s="2"/>
+      <c r="B85" s="10"/>
+      <c r="C85" s="2"/>
+      <c r="D85" s="5"/>
+      <c r="E85" s="2"/>
+    </row>
+    <row r="86" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A86" s="2"/>
+      <c r="B86" s="10"/>
+      <c r="C86" s="2"/>
+      <c r="D86" s="5"/>
+      <c r="E86" s="2"/>
+    </row>
+    <row r="87" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A87" s="2"/>
+      <c r="B87" s="10"/>
+      <c r="C87" s="2"/>
+      <c r="D87" s="5"/>
+      <c r="E87" s="2"/>
+    </row>
+    <row r="88" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A88" s="2"/>
+      <c r="B88" s="10"/>
+      <c r="C88" s="2"/>
+      <c r="D88" s="5"/>
+      <c r="E88" s="2"/>
+    </row>
+    <row r="89" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A89" s="2"/>
+      <c r="B89" s="10"/>
+      <c r="C89" s="2"/>
+      <c r="D89" s="5"/>
+      <c r="E89" s="2"/>
+    </row>
+    <row r="90" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A90" s="2"/>
+      <c r="B90" s="10"/>
+      <c r="C90" s="2"/>
+      <c r="D90" s="5"/>
+      <c r="E90" s="2"/>
+    </row>
+    <row r="91" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A91" s="2"/>
+      <c r="B91" s="10"/>
+      <c r="C91" s="2"/>
+      <c r="D91" s="5"/>
+      <c r="E91" s="2"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <dataValidations count="4">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C9:C249" xr:uid="{F5616ACF-4579-4F51-98EB-3A42CAF53755}">
+      <formula1>1</formula1>
+      <formula2>30</formula2>
+    </dataValidation>
+    <dataValidation type="textLength" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B3" xr:uid="{B3C00A21-6C3B-4BF1-AED1-57B07B687140}">
+      <formula1>3</formula1>
+      <formula2>25</formula2>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A5" xr:uid="{CD539E6C-2947-4534-8D36-C6FE16F17852}">
+      <formula1>"English, Computer, Science, Math, Geography, History, General Knowledge, Social Studies, Life Skills"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A3" xr:uid="{F882A79E-2D54-4987-95F5-500816EFE882}">
+      <formula1>"KG, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, Other"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>